<commit_message>
🔄 Update: 23 Mar 2026 12:12 UTC
</commit_message>
<xml_diff>
--- a/docs/africa_fuel_prices.xlsx
+++ b/docs/africa_fuel_prices.xlsx
@@ -1314,7 +1314,7 @@
     <row r="3" ht="18" customHeight="1">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Updated: 23 March 2026  |  11:26 UTC  ·  54 Countries  ·  5 Regions  ·  Prices in USD/L and Local Currency/L  ·  Sources: GlobalPetrolPrices · OPEC · World Bank</t>
+          <t>Updated: 23 March 2026  |  12:12 UTC  ·  54 Countries  ·  5 Regions  ·  Prices in USD/L and Local Currency/L  ·  Sources: GlobalPetrolPrices · OPEC · World Bank</t>
         </is>
       </c>
     </row>
@@ -1564,7 +1564,7 @@
       </c>
       <c r="R11" s="23" t="inlineStr">
         <is>
-          <t>2026-03-23 11:26 UTC</t>
+          <t>2026-03-23 12:12 UTC</t>
         </is>
       </c>
     </row>
@@ -1627,7 +1627,7 @@
       </c>
       <c r="R12" s="32" t="inlineStr">
         <is>
-          <t>2026-03-23 11:26 UTC</t>
+          <t>2026-03-23 12:12 UTC</t>
         </is>
       </c>
     </row>
@@ -1690,7 +1690,7 @@
       </c>
       <c r="R13" s="23" t="inlineStr">
         <is>
-          <t>2026-03-23 11:26 UTC</t>
+          <t>2026-03-23 12:12 UTC</t>
         </is>
       </c>
     </row>
@@ -1753,7 +1753,7 @@
       </c>
       <c r="R14" s="32" t="inlineStr">
         <is>
-          <t>2026-03-23 11:26 UTC</t>
+          <t>2026-03-23 12:12 UTC</t>
         </is>
       </c>
     </row>
@@ -1816,7 +1816,7 @@
       </c>
       <c r="R15" s="23" t="inlineStr">
         <is>
-          <t>2026-03-23 11:26 UTC</t>
+          <t>2026-03-23 12:12 UTC</t>
         </is>
       </c>
     </row>
@@ -1879,7 +1879,7 @@
       </c>
       <c r="R16" s="32" t="inlineStr">
         <is>
-          <t>2026-03-23 11:26 UTC</t>
+          <t>2026-03-23 12:12 UTC</t>
         </is>
       </c>
     </row>
@@ -1942,7 +1942,7 @@
       </c>
       <c r="R17" s="23" t="inlineStr">
         <is>
-          <t>2026-03-23 11:26 UTC</t>
+          <t>2026-03-23 12:12 UTC</t>
         </is>
       </c>
     </row>
@@ -2005,7 +2005,7 @@
       </c>
       <c r="R18" s="32" t="inlineStr">
         <is>
-          <t>2026-03-23 11:26 UTC</t>
+          <t>2026-03-23 12:12 UTC</t>
         </is>
       </c>
     </row>
@@ -2068,7 +2068,7 @@
       </c>
       <c r="R19" s="23" t="inlineStr">
         <is>
-          <t>2026-03-23 11:26 UTC</t>
+          <t>2026-03-23 12:12 UTC</t>
         </is>
       </c>
     </row>
@@ -2131,7 +2131,7 @@
       </c>
       <c r="R20" s="32" t="inlineStr">
         <is>
-          <t>2026-03-23 11:26 UTC</t>
+          <t>2026-03-23 12:12 UTC</t>
         </is>
       </c>
     </row>
@@ -2194,7 +2194,7 @@
       </c>
       <c r="R21" s="23" t="inlineStr">
         <is>
-          <t>2026-03-23 11:26 UTC</t>
+          <t>2026-03-23 12:12 UTC</t>
         </is>
       </c>
     </row>
@@ -2257,7 +2257,7 @@
       </c>
       <c r="R22" s="32" t="inlineStr">
         <is>
-          <t>2026-03-23 11:26 UTC</t>
+          <t>2026-03-23 12:12 UTC</t>
         </is>
       </c>
     </row>
@@ -2320,7 +2320,7 @@
       </c>
       <c r="R23" s="23" t="inlineStr">
         <is>
-          <t>2026-03-23 11:26 UTC</t>
+          <t>2026-03-23 12:12 UTC</t>
         </is>
       </c>
     </row>
@@ -2383,7 +2383,7 @@
       </c>
       <c r="R24" s="32" t="inlineStr">
         <is>
-          <t>2026-03-23 11:26 UTC</t>
+          <t>2026-03-23 12:12 UTC</t>
         </is>
       </c>
     </row>
@@ -2446,7 +2446,7 @@
       </c>
       <c r="R25" s="23" t="inlineStr">
         <is>
-          <t>2026-03-23 11:26 UTC</t>
+          <t>2026-03-23 12:12 UTC</t>
         </is>
       </c>
     </row>
@@ -2509,7 +2509,7 @@
       </c>
       <c r="R26" s="32" t="inlineStr">
         <is>
-          <t>2026-03-23 11:26 UTC</t>
+          <t>2026-03-23 12:12 UTC</t>
         </is>
       </c>
     </row>
@@ -2572,7 +2572,7 @@
       </c>
       <c r="R27" s="23" t="inlineStr">
         <is>
-          <t>2026-03-23 11:26 UTC</t>
+          <t>2026-03-23 12:12 UTC</t>
         </is>
       </c>
     </row>
@@ -2635,7 +2635,7 @@
       </c>
       <c r="R28" s="32" t="inlineStr">
         <is>
-          <t>2026-03-23 11:26 UTC</t>
+          <t>2026-03-23 12:12 UTC</t>
         </is>
       </c>
     </row>
@@ -2698,7 +2698,7 @@
       </c>
       <c r="R29" s="23" t="inlineStr">
         <is>
-          <t>2026-03-23 11:26 UTC</t>
+          <t>2026-03-23 12:12 UTC</t>
         </is>
       </c>
     </row>
@@ -2761,7 +2761,7 @@
       </c>
       <c r="R30" s="32" t="inlineStr">
         <is>
-          <t>2026-03-23 11:26 UTC</t>
+          <t>2026-03-23 12:12 UTC</t>
         </is>
       </c>
     </row>
@@ -2824,7 +2824,7 @@
       </c>
       <c r="R31" s="23" t="inlineStr">
         <is>
-          <t>2026-03-23 11:26 UTC</t>
+          <t>2026-03-23 12:12 UTC</t>
         </is>
       </c>
     </row>
@@ -2887,7 +2887,7 @@
       </c>
       <c r="R32" s="32" t="inlineStr">
         <is>
-          <t>2026-03-23 11:26 UTC</t>
+          <t>2026-03-23 12:12 UTC</t>
         </is>
       </c>
     </row>
@@ -2950,7 +2950,7 @@
       </c>
       <c r="R33" s="23" t="inlineStr">
         <is>
-          <t>2026-03-23 11:26 UTC</t>
+          <t>2026-03-23 12:12 UTC</t>
         </is>
       </c>
     </row>
@@ -3013,7 +3013,7 @@
       </c>
       <c r="R34" s="32" t="inlineStr">
         <is>
-          <t>2026-03-23 11:26 UTC</t>
+          <t>2026-03-23 12:12 UTC</t>
         </is>
       </c>
     </row>
@@ -3076,7 +3076,7 @@
       </c>
       <c r="R35" s="23" t="inlineStr">
         <is>
-          <t>2026-03-23 11:26 UTC</t>
+          <t>2026-03-23 12:12 UTC</t>
         </is>
       </c>
     </row>
@@ -3139,7 +3139,7 @@
       </c>
       <c r="R36" s="32" t="inlineStr">
         <is>
-          <t>2026-03-23 11:26 UTC</t>
+          <t>2026-03-23 12:12 UTC</t>
         </is>
       </c>
     </row>
@@ -3202,7 +3202,7 @@
       </c>
       <c r="R37" s="23" t="inlineStr">
         <is>
-          <t>2026-03-23 11:26 UTC</t>
+          <t>2026-03-23 12:12 UTC</t>
         </is>
       </c>
     </row>
@@ -3265,7 +3265,7 @@
       </c>
       <c r="R38" s="32" t="inlineStr">
         <is>
-          <t>2026-03-23 11:26 UTC</t>
+          <t>2026-03-23 12:12 UTC</t>
         </is>
       </c>
     </row>
@@ -3328,7 +3328,7 @@
       </c>
       <c r="R39" s="23" t="inlineStr">
         <is>
-          <t>2026-03-23 11:26 UTC</t>
+          <t>2026-03-23 12:12 UTC</t>
         </is>
       </c>
     </row>
@@ -3391,7 +3391,7 @@
       </c>
       <c r="R40" s="32" t="inlineStr">
         <is>
-          <t>2026-03-23 11:26 UTC</t>
+          <t>2026-03-23 12:12 UTC</t>
         </is>
       </c>
     </row>
@@ -3454,7 +3454,7 @@
       </c>
       <c r="R41" s="23" t="inlineStr">
         <is>
-          <t>2026-03-23 11:26 UTC</t>
+          <t>2026-03-23 12:12 UTC</t>
         </is>
       </c>
     </row>
@@ -3517,7 +3517,7 @@
       </c>
       <c r="R42" s="32" t="inlineStr">
         <is>
-          <t>2026-03-23 11:26 UTC</t>
+          <t>2026-03-23 12:12 UTC</t>
         </is>
       </c>
     </row>
@@ -3580,7 +3580,7 @@
       </c>
       <c r="R43" s="23" t="inlineStr">
         <is>
-          <t>2026-03-23 11:26 UTC</t>
+          <t>2026-03-23 12:12 UTC</t>
         </is>
       </c>
     </row>
@@ -3643,7 +3643,7 @@
       </c>
       <c r="R44" s="32" t="inlineStr">
         <is>
-          <t>2026-03-23 11:26 UTC</t>
+          <t>2026-03-23 12:12 UTC</t>
         </is>
       </c>
     </row>
@@ -3706,7 +3706,7 @@
       </c>
       <c r="R45" s="23" t="inlineStr">
         <is>
-          <t>2026-03-23 11:26 UTC</t>
+          <t>2026-03-23 12:12 UTC</t>
         </is>
       </c>
     </row>
@@ -3769,7 +3769,7 @@
       </c>
       <c r="R46" s="32" t="inlineStr">
         <is>
-          <t>2026-03-23 11:26 UTC</t>
+          <t>2026-03-23 12:12 UTC</t>
         </is>
       </c>
     </row>
@@ -3832,7 +3832,7 @@
       </c>
       <c r="R47" s="23" t="inlineStr">
         <is>
-          <t>2026-03-23 11:26 UTC</t>
+          <t>2026-03-23 12:12 UTC</t>
         </is>
       </c>
     </row>
@@ -3895,7 +3895,7 @@
       </c>
       <c r="R48" s="32" t="inlineStr">
         <is>
-          <t>2026-03-23 11:26 UTC</t>
+          <t>2026-03-23 12:12 UTC</t>
         </is>
       </c>
     </row>
@@ -3958,7 +3958,7 @@
       </c>
       <c r="R49" s="23" t="inlineStr">
         <is>
-          <t>2026-03-23 11:26 UTC</t>
+          <t>2026-03-23 12:12 UTC</t>
         </is>
       </c>
     </row>
@@ -4021,7 +4021,7 @@
       </c>
       <c r="R50" s="32" t="inlineStr">
         <is>
-          <t>2026-03-23 11:26 UTC</t>
+          <t>2026-03-23 12:12 UTC</t>
         </is>
       </c>
     </row>
@@ -4084,7 +4084,7 @@
       </c>
       <c r="R51" s="23" t="inlineStr">
         <is>
-          <t>2026-03-23 11:26 UTC</t>
+          <t>2026-03-23 12:12 UTC</t>
         </is>
       </c>
     </row>
@@ -4147,7 +4147,7 @@
       </c>
       <c r="R52" s="32" t="inlineStr">
         <is>
-          <t>2026-03-23 11:26 UTC</t>
+          <t>2026-03-23 12:12 UTC</t>
         </is>
       </c>
     </row>
@@ -14476,7 +14476,7 @@
       </c>
       <c r="C4" s="70" t="inlineStr">
         <is>
-          <t>23 March 2026 — 11:26 UTC</t>
+          <t>23 March 2026 — 12:12 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
🔄 Update: 23 Mar 2026 16:23 UTC
</commit_message>
<xml_diff>
--- a/docs/africa_fuel_prices.xlsx
+++ b/docs/africa_fuel_prices.xlsx
@@ -1314,7 +1314,7 @@
     <row r="3" ht="18" customHeight="1">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Updated: 23 March 2026  |  12:12 UTC  ·  54 Countries  ·  5 Regions  ·  Prices in USD/L and Local Currency/L  ·  Sources: GlobalPetrolPrices · OPEC · World Bank</t>
+          <t>Updated: 23 March 2026  |  16:23 UTC  ·  54 Countries  ·  5 Regions  ·  Prices in USD/L and Local Currency/L  ·  Sources: GlobalPetrolPrices · OPEC · World Bank</t>
         </is>
       </c>
     </row>
@@ -1564,7 +1564,7 @@
       </c>
       <c r="R11" s="23" t="inlineStr">
         <is>
-          <t>2026-03-23 12:12 UTC</t>
+          <t>2026-03-23 16:23 UTC</t>
         </is>
       </c>
     </row>
@@ -1627,7 +1627,7 @@
       </c>
       <c r="R12" s="32" t="inlineStr">
         <is>
-          <t>2026-03-23 12:12 UTC</t>
+          <t>2026-03-23 16:23 UTC</t>
         </is>
       </c>
     </row>
@@ -1690,7 +1690,7 @@
       </c>
       <c r="R13" s="23" t="inlineStr">
         <is>
-          <t>2026-03-23 12:12 UTC</t>
+          <t>2026-03-23 16:23 UTC</t>
         </is>
       </c>
     </row>
@@ -1753,7 +1753,7 @@
       </c>
       <c r="R14" s="32" t="inlineStr">
         <is>
-          <t>2026-03-23 12:12 UTC</t>
+          <t>2026-03-23 16:23 UTC</t>
         </is>
       </c>
     </row>
@@ -1816,7 +1816,7 @@
       </c>
       <c r="R15" s="23" t="inlineStr">
         <is>
-          <t>2026-03-23 12:12 UTC</t>
+          <t>2026-03-23 16:23 UTC</t>
         </is>
       </c>
     </row>
@@ -1879,7 +1879,7 @@
       </c>
       <c r="R16" s="32" t="inlineStr">
         <is>
-          <t>2026-03-23 12:12 UTC</t>
+          <t>2026-03-23 16:23 UTC</t>
         </is>
       </c>
     </row>
@@ -1942,7 +1942,7 @@
       </c>
       <c r="R17" s="23" t="inlineStr">
         <is>
-          <t>2026-03-23 12:12 UTC</t>
+          <t>2026-03-23 16:23 UTC</t>
         </is>
       </c>
     </row>
@@ -2005,7 +2005,7 @@
       </c>
       <c r="R18" s="32" t="inlineStr">
         <is>
-          <t>2026-03-23 12:12 UTC</t>
+          <t>2026-03-23 16:23 UTC</t>
         </is>
       </c>
     </row>
@@ -2068,7 +2068,7 @@
       </c>
       <c r="R19" s="23" t="inlineStr">
         <is>
-          <t>2026-03-23 12:12 UTC</t>
+          <t>2026-03-23 16:23 UTC</t>
         </is>
       </c>
     </row>
@@ -2131,7 +2131,7 @@
       </c>
       <c r="R20" s="32" t="inlineStr">
         <is>
-          <t>2026-03-23 12:12 UTC</t>
+          <t>2026-03-23 16:23 UTC</t>
         </is>
       </c>
     </row>
@@ -2194,7 +2194,7 @@
       </c>
       <c r="R21" s="23" t="inlineStr">
         <is>
-          <t>2026-03-23 12:12 UTC</t>
+          <t>2026-03-23 16:23 UTC</t>
         </is>
       </c>
     </row>
@@ -2257,7 +2257,7 @@
       </c>
       <c r="R22" s="32" t="inlineStr">
         <is>
-          <t>2026-03-23 12:12 UTC</t>
+          <t>2026-03-23 16:23 UTC</t>
         </is>
       </c>
     </row>
@@ -2320,7 +2320,7 @@
       </c>
       <c r="R23" s="23" t="inlineStr">
         <is>
-          <t>2026-03-23 12:12 UTC</t>
+          <t>2026-03-23 16:23 UTC</t>
         </is>
       </c>
     </row>
@@ -2383,7 +2383,7 @@
       </c>
       <c r="R24" s="32" t="inlineStr">
         <is>
-          <t>2026-03-23 12:12 UTC</t>
+          <t>2026-03-23 16:23 UTC</t>
         </is>
       </c>
     </row>
@@ -2446,7 +2446,7 @@
       </c>
       <c r="R25" s="23" t="inlineStr">
         <is>
-          <t>2026-03-23 12:12 UTC</t>
+          <t>2026-03-23 16:23 UTC</t>
         </is>
       </c>
     </row>
@@ -2509,7 +2509,7 @@
       </c>
       <c r="R26" s="32" t="inlineStr">
         <is>
-          <t>2026-03-23 12:12 UTC</t>
+          <t>2026-03-23 16:23 UTC</t>
         </is>
       </c>
     </row>
@@ -2572,7 +2572,7 @@
       </c>
       <c r="R27" s="23" t="inlineStr">
         <is>
-          <t>2026-03-23 12:12 UTC</t>
+          <t>2026-03-23 16:23 UTC</t>
         </is>
       </c>
     </row>
@@ -2635,7 +2635,7 @@
       </c>
       <c r="R28" s="32" t="inlineStr">
         <is>
-          <t>2026-03-23 12:12 UTC</t>
+          <t>2026-03-23 16:23 UTC</t>
         </is>
       </c>
     </row>
@@ -2698,7 +2698,7 @@
       </c>
       <c r="R29" s="23" t="inlineStr">
         <is>
-          <t>2026-03-23 12:12 UTC</t>
+          <t>2026-03-23 16:23 UTC</t>
         </is>
       </c>
     </row>
@@ -2761,7 +2761,7 @@
       </c>
       <c r="R30" s="32" t="inlineStr">
         <is>
-          <t>2026-03-23 12:12 UTC</t>
+          <t>2026-03-23 16:23 UTC</t>
         </is>
       </c>
     </row>
@@ -2824,7 +2824,7 @@
       </c>
       <c r="R31" s="23" t="inlineStr">
         <is>
-          <t>2026-03-23 12:12 UTC</t>
+          <t>2026-03-23 16:23 UTC</t>
         </is>
       </c>
     </row>
@@ -2887,7 +2887,7 @@
       </c>
       <c r="R32" s="32" t="inlineStr">
         <is>
-          <t>2026-03-23 12:12 UTC</t>
+          <t>2026-03-23 16:23 UTC</t>
         </is>
       </c>
     </row>
@@ -2950,7 +2950,7 @@
       </c>
       <c r="R33" s="23" t="inlineStr">
         <is>
-          <t>2026-03-23 12:12 UTC</t>
+          <t>2026-03-23 16:23 UTC</t>
         </is>
       </c>
     </row>
@@ -3013,7 +3013,7 @@
       </c>
       <c r="R34" s="32" t="inlineStr">
         <is>
-          <t>2026-03-23 12:12 UTC</t>
+          <t>2026-03-23 16:23 UTC</t>
         </is>
       </c>
     </row>
@@ -3076,7 +3076,7 @@
       </c>
       <c r="R35" s="23" t="inlineStr">
         <is>
-          <t>2026-03-23 12:12 UTC</t>
+          <t>2026-03-23 16:23 UTC</t>
         </is>
       </c>
     </row>
@@ -3139,7 +3139,7 @@
       </c>
       <c r="R36" s="32" t="inlineStr">
         <is>
-          <t>2026-03-23 12:12 UTC</t>
+          <t>2026-03-23 16:23 UTC</t>
         </is>
       </c>
     </row>
@@ -3202,7 +3202,7 @@
       </c>
       <c r="R37" s="23" t="inlineStr">
         <is>
-          <t>2026-03-23 12:12 UTC</t>
+          <t>2026-03-23 16:23 UTC</t>
         </is>
       </c>
     </row>
@@ -3265,7 +3265,7 @@
       </c>
       <c r="R38" s="32" t="inlineStr">
         <is>
-          <t>2026-03-23 12:12 UTC</t>
+          <t>2026-03-23 16:23 UTC</t>
         </is>
       </c>
     </row>
@@ -3328,7 +3328,7 @@
       </c>
       <c r="R39" s="23" t="inlineStr">
         <is>
-          <t>2026-03-23 12:12 UTC</t>
+          <t>2026-03-23 16:23 UTC</t>
         </is>
       </c>
     </row>
@@ -3391,7 +3391,7 @@
       </c>
       <c r="R40" s="32" t="inlineStr">
         <is>
-          <t>2026-03-23 12:12 UTC</t>
+          <t>2026-03-23 16:23 UTC</t>
         </is>
       </c>
     </row>
@@ -3454,7 +3454,7 @@
       </c>
       <c r="R41" s="23" t="inlineStr">
         <is>
-          <t>2026-03-23 12:12 UTC</t>
+          <t>2026-03-23 16:23 UTC</t>
         </is>
       </c>
     </row>
@@ -3517,7 +3517,7 @@
       </c>
       <c r="R42" s="32" t="inlineStr">
         <is>
-          <t>2026-03-23 12:12 UTC</t>
+          <t>2026-03-23 16:23 UTC</t>
         </is>
       </c>
     </row>
@@ -3580,7 +3580,7 @@
       </c>
       <c r="R43" s="23" t="inlineStr">
         <is>
-          <t>2026-03-23 12:12 UTC</t>
+          <t>2026-03-23 16:23 UTC</t>
         </is>
       </c>
     </row>
@@ -3643,7 +3643,7 @@
       </c>
       <c r="R44" s="32" t="inlineStr">
         <is>
-          <t>2026-03-23 12:12 UTC</t>
+          <t>2026-03-23 16:23 UTC</t>
         </is>
       </c>
     </row>
@@ -3706,7 +3706,7 @@
       </c>
       <c r="R45" s="23" t="inlineStr">
         <is>
-          <t>2026-03-23 12:12 UTC</t>
+          <t>2026-03-23 16:23 UTC</t>
         </is>
       </c>
     </row>
@@ -3769,7 +3769,7 @@
       </c>
       <c r="R46" s="32" t="inlineStr">
         <is>
-          <t>2026-03-23 12:12 UTC</t>
+          <t>2026-03-23 16:23 UTC</t>
         </is>
       </c>
     </row>
@@ -3832,7 +3832,7 @@
       </c>
       <c r="R47" s="23" t="inlineStr">
         <is>
-          <t>2026-03-23 12:12 UTC</t>
+          <t>2026-03-23 16:23 UTC</t>
         </is>
       </c>
     </row>
@@ -3895,7 +3895,7 @@
       </c>
       <c r="R48" s="32" t="inlineStr">
         <is>
-          <t>2026-03-23 12:12 UTC</t>
+          <t>2026-03-23 16:23 UTC</t>
         </is>
       </c>
     </row>
@@ -3958,7 +3958,7 @@
       </c>
       <c r="R49" s="23" t="inlineStr">
         <is>
-          <t>2026-03-23 12:12 UTC</t>
+          <t>2026-03-23 16:23 UTC</t>
         </is>
       </c>
     </row>
@@ -4021,7 +4021,7 @@
       </c>
       <c r="R50" s="32" t="inlineStr">
         <is>
-          <t>2026-03-23 12:12 UTC</t>
+          <t>2026-03-23 16:23 UTC</t>
         </is>
       </c>
     </row>
@@ -4084,7 +4084,7 @@
       </c>
       <c r="R51" s="23" t="inlineStr">
         <is>
-          <t>2026-03-23 12:12 UTC</t>
+          <t>2026-03-23 16:23 UTC</t>
         </is>
       </c>
     </row>
@@ -4147,7 +4147,7 @@
       </c>
       <c r="R52" s="32" t="inlineStr">
         <is>
-          <t>2026-03-23 12:12 UTC</t>
+          <t>2026-03-23 16:23 UTC</t>
         </is>
       </c>
     </row>
@@ -14476,7 +14476,7 @@
       </c>
       <c r="C4" s="70" t="inlineStr">
         <is>
-          <t>23 March 2026 — 12:12 UTC</t>
+          <t>23 March 2026 — 16:23 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
🔄 Update: 24 Mar 2026 08:19 UTC
</commit_message>
<xml_diff>
--- a/docs/africa_fuel_prices.xlsx
+++ b/docs/africa_fuel_prices.xlsx
@@ -1314,7 +1314,7 @@
     <row r="3" ht="18" customHeight="1">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Updated: 24 March 2026  |  06:59 UTC  ·  54 Countries  ·  5 Regions  ·  Prices in USD/L and Local Currency/L  ·  Sources: GlobalPetrolPrices · OPEC · World Bank</t>
+          <t>Updated: 24 March 2026  |  08:19 UTC  ·  54 Countries  ·  5 Regions  ·  Prices in USD/L and Local Currency/L  ·  Sources: GlobalPetrolPrices · OPEC · World Bank</t>
         </is>
       </c>
     </row>
@@ -1564,7 +1564,7 @@
       </c>
       <c r="R11" s="23" t="inlineStr">
         <is>
-          <t>2026-03-24 06:59 UTC</t>
+          <t>2026-03-24 08:19 UTC</t>
         </is>
       </c>
     </row>
@@ -1627,7 +1627,7 @@
       </c>
       <c r="R12" s="32" t="inlineStr">
         <is>
-          <t>2026-03-24 06:59 UTC</t>
+          <t>2026-03-24 08:19 UTC</t>
         </is>
       </c>
     </row>
@@ -1690,7 +1690,7 @@
       </c>
       <c r="R13" s="23" t="inlineStr">
         <is>
-          <t>2026-03-24 06:59 UTC</t>
+          <t>2026-03-24 08:19 UTC</t>
         </is>
       </c>
     </row>
@@ -1753,7 +1753,7 @@
       </c>
       <c r="R14" s="32" t="inlineStr">
         <is>
-          <t>2026-03-24 06:59 UTC</t>
+          <t>2026-03-24 08:19 UTC</t>
         </is>
       </c>
     </row>
@@ -1816,7 +1816,7 @@
       </c>
       <c r="R15" s="23" t="inlineStr">
         <is>
-          <t>2026-03-24 06:59 UTC</t>
+          <t>2026-03-24 08:19 UTC</t>
         </is>
       </c>
     </row>
@@ -1879,7 +1879,7 @@
       </c>
       <c r="R16" s="32" t="inlineStr">
         <is>
-          <t>2026-03-24 06:59 UTC</t>
+          <t>2026-03-24 08:19 UTC</t>
         </is>
       </c>
     </row>
@@ -1942,7 +1942,7 @@
       </c>
       <c r="R17" s="23" t="inlineStr">
         <is>
-          <t>2026-03-24 06:59 UTC</t>
+          <t>2026-03-24 08:19 UTC</t>
         </is>
       </c>
     </row>
@@ -2005,7 +2005,7 @@
       </c>
       <c r="R18" s="32" t="inlineStr">
         <is>
-          <t>2026-03-24 06:59 UTC</t>
+          <t>2026-03-24 08:19 UTC</t>
         </is>
       </c>
     </row>
@@ -2068,7 +2068,7 @@
       </c>
       <c r="R19" s="23" t="inlineStr">
         <is>
-          <t>2026-03-24 06:59 UTC</t>
+          <t>2026-03-24 08:19 UTC</t>
         </is>
       </c>
     </row>
@@ -2131,7 +2131,7 @@
       </c>
       <c r="R20" s="32" t="inlineStr">
         <is>
-          <t>2026-03-24 06:59 UTC</t>
+          <t>2026-03-24 08:19 UTC</t>
         </is>
       </c>
     </row>
@@ -2194,7 +2194,7 @@
       </c>
       <c r="R21" s="23" t="inlineStr">
         <is>
-          <t>2026-03-24 06:59 UTC</t>
+          <t>2026-03-24 08:19 UTC</t>
         </is>
       </c>
     </row>
@@ -2257,7 +2257,7 @@
       </c>
       <c r="R22" s="32" t="inlineStr">
         <is>
-          <t>2026-03-24 06:59 UTC</t>
+          <t>2026-03-24 08:19 UTC</t>
         </is>
       </c>
     </row>
@@ -2320,7 +2320,7 @@
       </c>
       <c r="R23" s="23" t="inlineStr">
         <is>
-          <t>2026-03-24 06:59 UTC</t>
+          <t>2026-03-24 08:19 UTC</t>
         </is>
       </c>
     </row>
@@ -2383,7 +2383,7 @@
       </c>
       <c r="R24" s="32" t="inlineStr">
         <is>
-          <t>2026-03-24 06:59 UTC</t>
+          <t>2026-03-24 08:19 UTC</t>
         </is>
       </c>
     </row>
@@ -2446,7 +2446,7 @@
       </c>
       <c r="R25" s="23" t="inlineStr">
         <is>
-          <t>2026-03-24 06:59 UTC</t>
+          <t>2026-03-24 08:19 UTC</t>
         </is>
       </c>
     </row>
@@ -2509,7 +2509,7 @@
       </c>
       <c r="R26" s="32" t="inlineStr">
         <is>
-          <t>2026-03-24 06:59 UTC</t>
+          <t>2026-03-24 08:19 UTC</t>
         </is>
       </c>
     </row>
@@ -2572,7 +2572,7 @@
       </c>
       <c r="R27" s="23" t="inlineStr">
         <is>
-          <t>2026-03-24 06:59 UTC</t>
+          <t>2026-03-24 08:19 UTC</t>
         </is>
       </c>
     </row>
@@ -2635,7 +2635,7 @@
       </c>
       <c r="R28" s="32" t="inlineStr">
         <is>
-          <t>2026-03-24 06:59 UTC</t>
+          <t>2026-03-24 08:19 UTC</t>
         </is>
       </c>
     </row>
@@ -2698,7 +2698,7 @@
       </c>
       <c r="R29" s="23" t="inlineStr">
         <is>
-          <t>2026-03-24 06:59 UTC</t>
+          <t>2026-03-24 08:19 UTC</t>
         </is>
       </c>
     </row>
@@ -2761,7 +2761,7 @@
       </c>
       <c r="R30" s="32" t="inlineStr">
         <is>
-          <t>2026-03-24 06:59 UTC</t>
+          <t>2026-03-24 08:19 UTC</t>
         </is>
       </c>
     </row>
@@ -2824,7 +2824,7 @@
       </c>
       <c r="R31" s="23" t="inlineStr">
         <is>
-          <t>2026-03-24 06:59 UTC</t>
+          <t>2026-03-24 08:19 UTC</t>
         </is>
       </c>
     </row>
@@ -2887,7 +2887,7 @@
       </c>
       <c r="R32" s="32" t="inlineStr">
         <is>
-          <t>2026-03-24 06:59 UTC</t>
+          <t>2026-03-24 08:19 UTC</t>
         </is>
       </c>
     </row>
@@ -2950,7 +2950,7 @@
       </c>
       <c r="R33" s="23" t="inlineStr">
         <is>
-          <t>2026-03-24 06:59 UTC</t>
+          <t>2026-03-24 08:19 UTC</t>
         </is>
       </c>
     </row>
@@ -3013,7 +3013,7 @@
       </c>
       <c r="R34" s="32" t="inlineStr">
         <is>
-          <t>2026-03-24 06:59 UTC</t>
+          <t>2026-03-24 08:19 UTC</t>
         </is>
       </c>
     </row>
@@ -3076,7 +3076,7 @@
       </c>
       <c r="R35" s="23" t="inlineStr">
         <is>
-          <t>2026-03-24 06:59 UTC</t>
+          <t>2026-03-24 08:19 UTC</t>
         </is>
       </c>
     </row>
@@ -3139,7 +3139,7 @@
       </c>
       <c r="R36" s="32" t="inlineStr">
         <is>
-          <t>2026-03-24 06:59 UTC</t>
+          <t>2026-03-24 08:19 UTC</t>
         </is>
       </c>
     </row>
@@ -3202,7 +3202,7 @@
       </c>
       <c r="R37" s="23" t="inlineStr">
         <is>
-          <t>2026-03-24 06:59 UTC</t>
+          <t>2026-03-24 08:19 UTC</t>
         </is>
       </c>
     </row>
@@ -3265,7 +3265,7 @@
       </c>
       <c r="R38" s="32" t="inlineStr">
         <is>
-          <t>2026-03-24 06:59 UTC</t>
+          <t>2026-03-24 08:19 UTC</t>
         </is>
       </c>
     </row>
@@ -3328,7 +3328,7 @@
       </c>
       <c r="R39" s="23" t="inlineStr">
         <is>
-          <t>2026-03-24 06:59 UTC</t>
+          <t>2026-03-24 08:19 UTC</t>
         </is>
       </c>
     </row>
@@ -3391,7 +3391,7 @@
       </c>
       <c r="R40" s="32" t="inlineStr">
         <is>
-          <t>2026-03-24 06:59 UTC</t>
+          <t>2026-03-24 08:19 UTC</t>
         </is>
       </c>
     </row>
@@ -3454,7 +3454,7 @@
       </c>
       <c r="R41" s="23" t="inlineStr">
         <is>
-          <t>2026-03-24 06:59 UTC</t>
+          <t>2026-03-24 08:19 UTC</t>
         </is>
       </c>
     </row>
@@ -3517,7 +3517,7 @@
       </c>
       <c r="R42" s="32" t="inlineStr">
         <is>
-          <t>2026-03-24 06:59 UTC</t>
+          <t>2026-03-24 08:19 UTC</t>
         </is>
       </c>
     </row>
@@ -3580,7 +3580,7 @@
       </c>
       <c r="R43" s="23" t="inlineStr">
         <is>
-          <t>2026-03-24 06:59 UTC</t>
+          <t>2026-03-24 08:19 UTC</t>
         </is>
       </c>
     </row>
@@ -3643,7 +3643,7 @@
       </c>
       <c r="R44" s="32" t="inlineStr">
         <is>
-          <t>2026-03-24 06:59 UTC</t>
+          <t>2026-03-24 08:19 UTC</t>
         </is>
       </c>
     </row>
@@ -3706,7 +3706,7 @@
       </c>
       <c r="R45" s="23" t="inlineStr">
         <is>
-          <t>2026-03-24 06:59 UTC</t>
+          <t>2026-03-24 08:19 UTC</t>
         </is>
       </c>
     </row>
@@ -3769,7 +3769,7 @@
       </c>
       <c r="R46" s="32" t="inlineStr">
         <is>
-          <t>2026-03-24 06:59 UTC</t>
+          <t>2026-03-24 08:19 UTC</t>
         </is>
       </c>
     </row>
@@ -3832,7 +3832,7 @@
       </c>
       <c r="R47" s="23" t="inlineStr">
         <is>
-          <t>2026-03-24 06:59 UTC</t>
+          <t>2026-03-24 08:19 UTC</t>
         </is>
       </c>
     </row>
@@ -3895,7 +3895,7 @@
       </c>
       <c r="R48" s="32" t="inlineStr">
         <is>
-          <t>2026-03-24 06:59 UTC</t>
+          <t>2026-03-24 08:19 UTC</t>
         </is>
       </c>
     </row>
@@ -3958,7 +3958,7 @@
       </c>
       <c r="R49" s="23" t="inlineStr">
         <is>
-          <t>2026-03-24 06:59 UTC</t>
+          <t>2026-03-24 08:19 UTC</t>
         </is>
       </c>
     </row>
@@ -4021,7 +4021,7 @@
       </c>
       <c r="R50" s="32" t="inlineStr">
         <is>
-          <t>2026-03-24 06:59 UTC</t>
+          <t>2026-03-24 08:19 UTC</t>
         </is>
       </c>
     </row>
@@ -4084,7 +4084,7 @@
       </c>
       <c r="R51" s="23" t="inlineStr">
         <is>
-          <t>2026-03-24 06:59 UTC</t>
+          <t>2026-03-24 08:19 UTC</t>
         </is>
       </c>
     </row>
@@ -4147,7 +4147,7 @@
       </c>
       <c r="R52" s="32" t="inlineStr">
         <is>
-          <t>2026-03-24 06:59 UTC</t>
+          <t>2026-03-24 08:19 UTC</t>
         </is>
       </c>
     </row>
@@ -14476,7 +14476,7 @@
       </c>
       <c r="C4" s="70" t="inlineStr">
         <is>
-          <t>24 March 2026 — 06:59 UTC</t>
+          <t>24 March 2026 — 08:19 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>